<commit_message>
Adjust data type validation structure
</commit_message>
<xml_diff>
--- a/docs/input_data_template.xlsx
+++ b/docs/input_data_template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="24334"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30430"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Q:\Projekte\3-152-24-HBl_PyFlex\2 Inhalte\10 Arbeitspaket 5\pyromof-non-tabular\docs\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\klima\Documents\pyromof\pyromof\docs\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B9C7A18C-E394-4A4D-813A-955050EDEE4A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D2FA899D-1C44-4B80-8E26-198C6BDA6981}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="3555" yWindow="-19170" windowWidth="23250" windowHeight="13890" xr2:uid="{46330B2F-E85C-4459-B76B-09B0963C0FC2}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{46330B2F-E85C-4459-B76B-09B0963C0FC2}"/>
   </bookViews>
   <sheets>
     <sheet name="general" sheetId="8" r:id="rId1"/>
@@ -50,7 +50,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="100" uniqueCount="61">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="119" uniqueCount="72">
   <si>
     <t>biomass</t>
   </si>
@@ -118,9 +118,6 @@
     <t>timeindex</t>
   </si>
   <si>
-    <t>b_heat_in</t>
-  </si>
-  <si>
     <t>pyrolysis</t>
   </si>
   <si>
@@ -233,6 +230,42 @@
   </si>
   <si>
     <t>nominal_capacity</t>
+  </si>
+  <si>
+    <t>min</t>
+  </si>
+  <si>
+    <t>max</t>
+  </si>
+  <si>
+    <t>total_availability</t>
+  </si>
+  <si>
+    <t>bus_in_1_alternative</t>
+  </si>
+  <si>
+    <t>bus_out_4</t>
+  </si>
+  <si>
+    <t>eff_out_1_mod</t>
+  </si>
+  <si>
+    <t>eff_out_2_mod</t>
+  </si>
+  <si>
+    <t>maximum_startups</t>
+  </si>
+  <si>
+    <t>initial_status</t>
+  </si>
+  <si>
+    <t>offset</t>
+  </si>
+  <si>
+    <t>charge_rate</t>
+  </si>
+  <si>
+    <t>b_biochar_pre_shift</t>
   </si>
 </sst>
 </file>
@@ -356,26 +389,19 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1"/>
+    <xf numFmtId="11" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Standard" xfId="0" builtinId="0"/>
@@ -394,9 +420,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office 2013 – 2022-Design">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 – 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -434,7 +460,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 – 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -540,7 +566,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 – 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -682,7 +708,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -691,19 +717,19 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6E7BD6BA-64D6-4557-B3A9-74A7028C0BF6}">
   <dimension ref="A1:B2"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
-    <row r="1" spans="1:2" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:2" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>6</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>30</v>
-      </c>
-    </row>
-    <row r="2" spans="1:2" x14ac:dyDescent="0.3">
-      <c r="A2" s="9" t="s">
         <v>29</v>
+      </c>
+    </row>
+    <row r="2" spans="1:2" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>28</v>
       </c>
       <c r="B2">
         <v>0.05</v>
@@ -717,15 +743,15 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3735438E-83E5-49C0-829C-45BC687683E5}">
-  <dimension ref="A1:I6"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:K4"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="22.6640625" customWidth="1"/>
-    <col min="3" max="3" width="14.109375" customWidth="1"/>
-    <col min="6" max="6" width="14.6640625" customWidth="1"/>
+    <col min="1" max="1" width="22.7109375" customWidth="1"/>
+    <col min="3" max="3" width="14.140625" customWidth="1"/>
+    <col min="8" max="8" width="14.7109375" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>6</v>
       </c>
@@ -736,93 +762,86 @@
         <v>3</v>
       </c>
       <c r="D1" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="E1" s="1" t="s">
-        <v>59</v>
-      </c>
       <c r="F1" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="J1" s="1" t="s">
         <v>24</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="K1" s="1" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="2" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>17</v>
+      </c>
+      <c r="B2" t="s">
+        <v>15</v>
+      </c>
+      <c r="H2">
+        <v>-1000</v>
+      </c>
+      <c r="I2" t="s">
+        <v>36</v>
+      </c>
+      <c r="K2" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="3" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>18</v>
+      </c>
+      <c r="B3" t="s">
+        <v>16</v>
+      </c>
+      <c r="D3">
+        <v>1000</v>
+      </c>
+      <c r="G3">
+        <v>0</v>
+      </c>
+      <c r="H3">
+        <v>-125</v>
+      </c>
+      <c r="I3" t="s">
+        <v>36</v>
+      </c>
+      <c r="K3" t="s">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="4" spans="1:11" x14ac:dyDescent="0.25">
+      <c r="A4" t="s">
+        <v>47</v>
+      </c>
+      <c r="B4" t="s">
+        <v>42</v>
+      </c>
+      <c r="H4">
+        <v>0</v>
+      </c>
+      <c r="I4" t="s">
         <v>34</v>
       </c>
-      <c r="H1" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="2" spans="1:9" s="11" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="11" t="s">
-        <v>17</v>
-      </c>
-      <c r="B2" s="11" t="s">
-        <v>15</v>
-      </c>
-      <c r="D2" s="14"/>
-      <c r="E2" s="14"/>
-      <c r="F2" s="14">
-        <v>-1000</v>
-      </c>
-      <c r="G2" s="11" t="s">
-        <v>37</v>
-      </c>
-      <c r="I2" s="11" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9" s="11" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="11" t="s">
-        <v>18</v>
-      </c>
-      <c r="B3" s="11" t="s">
-        <v>16</v>
-      </c>
-      <c r="D3" s="14">
-        <v>1000</v>
-      </c>
-      <c r="E3" s="14">
-        <v>0</v>
-      </c>
-      <c r="F3" s="14">
-        <v>-125</v>
-      </c>
-      <c r="G3" s="11" t="s">
-        <v>37</v>
-      </c>
-      <c r="I3" s="11" t="s">
-        <v>58</v>
-      </c>
-    </row>
-    <row r="4" spans="1:9" s="11" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="11" t="s">
-        <v>48</v>
-      </c>
-      <c r="B4" s="11" t="s">
-        <v>43</v>
-      </c>
-      <c r="D4" s="14"/>
-      <c r="E4" s="14"/>
-      <c r="F4" s="14">
-        <v>0</v>
-      </c>
-      <c r="G4" s="11" t="s">
-        <v>35</v>
-      </c>
-      <c r="I4" s="11" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="D5" s="3"/>
-      <c r="E5" s="3"/>
-      <c r="F5" s="3"/>
-    </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.3">
-      <c r="F6" s="3"/>
-      <c r="I6" s="11"/>
+      <c r="K4" t="s">
+        <v>56</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
@@ -832,13 +851,13 @@
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{E07A0DDF-6A46-4B4C-A939-9103456CFEB0}">
-  <dimension ref="A1:I3"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:N3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="6" max="7" width="13.88671875" customWidth="1"/>
+    <col min="11" max="12" width="13.85546875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:14" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>6</v>
       </c>
@@ -849,68 +868,91 @@
         <v>3</v>
       </c>
       <c r="D1" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="F1" s="1" t="s">
         <v>60</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="G1" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>23</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="2" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A2" t="s">
+        <v>0</v>
+      </c>
+      <c r="B2" t="s">
+        <v>2</v>
+      </c>
+      <c r="D2">
+        <v>1000000000000000</v>
+      </c>
+      <c r="E2">
+        <v>800</v>
+      </c>
+      <c r="J2" t="s">
+        <v>35</v>
+      </c>
+      <c r="K2">
+        <v>250</v>
+      </c>
+      <c r="L2" t="s">
+        <v>36</v>
+      </c>
+      <c r="N2" t="s">
+        <v>56</v>
+      </c>
+    </row>
+    <row r="3" spans="1:14" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
+        <v>25</v>
+      </c>
+      <c r="B3" t="s">
+        <v>32</v>
+      </c>
+      <c r="D3" s="11">
+        <v>100000000000</v>
+      </c>
+      <c r="E3" s="11"/>
+      <c r="F3" s="11"/>
+      <c r="G3" s="11"/>
+      <c r="H3" s="11"/>
+      <c r="I3" s="11"/>
+      <c r="J3" t="s">
+        <v>26</v>
+      </c>
+      <c r="K3">
+        <v>10000000</v>
+      </c>
+      <c r="L3" t="s">
         <v>34</v>
       </c>
-      <c r="F1" s="1" t="s">
-        <v>24</v>
-      </c>
-      <c r="G1" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="2" spans="1:9" s="11" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="11" t="s">
-        <v>0</v>
-      </c>
-      <c r="B2" s="11" t="s">
-        <v>2</v>
-      </c>
-      <c r="D2" s="11">
-        <v>1000000000000000</v>
-      </c>
-      <c r="E2" s="11" t="s">
-        <v>36</v>
-      </c>
-      <c r="F2" s="14">
-        <v>250</v>
-      </c>
-      <c r="G2" s="11" t="s">
-        <v>37</v>
-      </c>
-      <c r="I2" s="11" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="3" spans="1:9" s="11" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="11" t="s">
-        <v>26</v>
-      </c>
-      <c r="B3" s="11" t="s">
-        <v>33</v>
-      </c>
-      <c r="D3" s="18">
-        <v>100000000000</v>
-      </c>
-      <c r="E3" s="11" t="s">
-        <v>27</v>
-      </c>
-      <c r="F3" s="14">
-        <v>10000000</v>
-      </c>
-      <c r="G3" s="11" t="s">
-        <v>35</v>
-      </c>
-      <c r="I3" s="11" t="s">
-        <v>57</v>
+      <c r="N3" t="s">
+        <v>56</v>
       </c>
     </row>
   </sheetData>
@@ -920,26 +962,24 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F6332336-4B3F-4107-8642-DA0628BBF2A2}">
-  <dimension ref="A1:Y4"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" outlineLevelCol="1" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:AG3"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" outlineLevelCol="1" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="16.44140625" customWidth="1"/>
-    <col min="2" max="2" width="12.6640625" customWidth="1"/>
-    <col min="4" max="4" width="16.88671875" customWidth="1"/>
-    <col min="7" max="7" width="9" customWidth="1"/>
-    <col min="8" max="8" width="7.44140625" customWidth="1" outlineLevel="1"/>
-    <col min="9" max="9" width="8" customWidth="1" outlineLevel="1"/>
-    <col min="10" max="10" width="10" customWidth="1" outlineLevel="1"/>
-    <col min="11" max="12" width="11.5546875" customWidth="1" outlineLevel="1"/>
-    <col min="13" max="13" width="9.109375" customWidth="1" outlineLevel="1"/>
-    <col min="14" max="17" width="8.6640625" customWidth="1" outlineLevel="1"/>
-    <col min="18" max="18" width="9.21875" customWidth="1"/>
-    <col min="19" max="20" width="11.5546875" customWidth="1" outlineLevel="1"/>
-    <col min="21" max="22" width="11.5546875" style="3" customWidth="1" outlineLevel="1"/>
-    <col min="23" max="23" width="11.5546875" customWidth="1" outlineLevel="1"/>
+    <col min="1" max="1" width="16.42578125" customWidth="1"/>
+    <col min="2" max="3" width="12.7109375" customWidth="1"/>
+    <col min="5" max="5" width="16.85546875" customWidth="1"/>
+    <col min="9" max="9" width="9" customWidth="1"/>
+    <col min="10" max="10" width="7.42578125" customWidth="1" outlineLevel="1"/>
+    <col min="11" max="11" width="8" customWidth="1" outlineLevel="1"/>
+    <col min="12" max="13" width="10" customWidth="1" outlineLevel="1"/>
+    <col min="14" max="15" width="11.5703125" customWidth="1" outlineLevel="1"/>
+    <col min="16" max="17" width="9.140625" customWidth="1" outlineLevel="1"/>
+    <col min="18" max="23" width="8.7109375" customWidth="1" outlineLevel="1"/>
+    <col min="24" max="24" width="9.28515625" customWidth="1"/>
+    <col min="25" max="31" width="11.5703125" customWidth="1" outlineLevel="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:25" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>6</v>
       </c>
@@ -947,226 +987,282 @@
         <v>7</v>
       </c>
       <c r="C1" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="D1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="E1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>64</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>59</v>
+      </c>
+      <c r="J1" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="K1" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="L1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="M1" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>52</v>
+      </c>
+      <c r="P1" s="7" t="s">
+        <v>14</v>
+      </c>
+      <c r="Q1" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="R1" s="1" t="s">
         <v>31</v>
       </c>
-      <c r="G1" s="12" t="s">
-        <v>60</v>
-      </c>
-      <c r="H1" s="1" t="s">
-        <v>11</v>
-      </c>
-      <c r="I1" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="J1" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="K1" s="1" t="s">
-        <v>52</v>
-      </c>
-      <c r="L1" s="1" t="s">
+      <c r="S1" s="1" t="s">
         <v>53</v>
       </c>
-      <c r="M1" s="8" t="s">
-        <v>14</v>
-      </c>
-      <c r="N1" s="10" t="s">
-        <v>32</v>
-      </c>
-      <c r="O1" s="10" t="s">
+      <c r="T1" s="1" t="s">
         <v>54</v>
       </c>
-      <c r="P1" s="10" t="s">
-        <v>55</v>
-      </c>
-      <c r="Q1" s="10" t="s">
-        <v>50</v>
-      </c>
-      <c r="R1" s="13" t="s">
-        <v>47</v>
-      </c>
-      <c r="S1" s="12" t="s">
-        <v>28</v>
-      </c>
-      <c r="T1" s="12" t="s">
+      <c r="U1" s="1" t="s">
+        <v>67</v>
+      </c>
+      <c r="V1" s="1" t="s">
+        <v>68</v>
+      </c>
+      <c r="W1" s="1" t="s">
+        <v>49</v>
+      </c>
+      <c r="X1" s="1" t="s">
+        <v>46</v>
+      </c>
+      <c r="Y1" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="Z1" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="AA1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="U1" s="12" t="s">
+      <c r="AB1" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="AC1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="V1" s="12" t="s">
-        <v>49</v>
-      </c>
-      <c r="W1" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="X1" s="12" t="s">
-        <v>44</v>
-      </c>
-      <c r="Y1" s="12" t="s">
-        <v>38</v>
-      </c>
-    </row>
-    <row r="2" spans="1:25" x14ac:dyDescent="0.3">
+      <c r="AD1" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="AE1" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="AF1" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="AG1" s="1" t="s">
+        <v>37</v>
+      </c>
+    </row>
+    <row r="2" spans="1:33" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="B2" t="s">
         <v>2</v>
       </c>
-      <c r="C2" t="s">
+      <c r="D2" t="s">
+        <v>32</v>
+      </c>
+      <c r="E2" t="s">
+        <v>71</v>
+      </c>
+      <c r="F2" t="s">
+        <v>42</v>
+      </c>
+      <c r="G2" t="s">
+        <v>15</v>
+      </c>
+      <c r="H2" t="s">
+        <v>16</v>
+      </c>
+      <c r="I2">
+        <v>1000</v>
+      </c>
+      <c r="J2">
+        <v>1</v>
+      </c>
+      <c r="K2">
+        <v>0.2</v>
+      </c>
+      <c r="L2">
+        <v>0.5</v>
+      </c>
+      <c r="M2">
+        <v>0.5</v>
+      </c>
+      <c r="N2">
+        <v>-0.25</v>
+      </c>
+      <c r="O2">
+        <v>0.1</v>
+      </c>
+      <c r="P2">
+        <v>0.5</v>
+      </c>
+      <c r="Q2">
+        <v>0.5</v>
+      </c>
+      <c r="R2">
+        <v>0.2</v>
+      </c>
+      <c r="S2">
+        <v>0.5</v>
+      </c>
+      <c r="T2">
+        <v>4</v>
+      </c>
+      <c r="U2">
+        <v>2</v>
+      </c>
+      <c r="V2">
+        <v>0</v>
+      </c>
+      <c r="W2">
+        <v>5</v>
+      </c>
+      <c r="X2">
+        <v>0.01</v>
+      </c>
+      <c r="Y2">
+        <v>1</v>
+      </c>
+      <c r="AA2">
+        <v>20</v>
+      </c>
+      <c r="AB2">
+        <v>59.5</v>
+      </c>
+      <c r="AC2">
+        <v>10000000</v>
+      </c>
+      <c r="AD2">
+        <v>0</v>
+      </c>
+      <c r="AF2" t="s">
+        <v>44</v>
+      </c>
+      <c r="AG2" t="s">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="3" spans="1:33" x14ac:dyDescent="0.25">
+      <c r="A3" t="s">
         <v>22</v>
       </c>
-      <c r="D2" t="s">
-        <v>33</v>
-      </c>
-      <c r="E2" t="s">
+      <c r="B3" t="s">
+        <v>2</v>
+      </c>
+      <c r="D3" t="s">
+        <v>32</v>
+      </c>
+      <c r="E3" t="s">
+        <v>71</v>
+      </c>
+      <c r="F3" t="s">
+        <v>42</v>
+      </c>
+      <c r="G3" t="s">
         <v>15</v>
       </c>
-      <c r="F2" t="s">
+      <c r="H3" t="s">
         <v>16</v>
       </c>
-      <c r="G2" s="3">
+      <c r="I3">
         <v>1000</v>
       </c>
-      <c r="H2">
+      <c r="J3">
         <v>1</v>
       </c>
-      <c r="I2">
-        <v>0.2</v>
-      </c>
-      <c r="J2">
-        <v>0.5</v>
-      </c>
-      <c r="K2">
+      <c r="K3">
+        <v>1</v>
+      </c>
+      <c r="L3">
+        <v>0.25700000000000001</v>
+      </c>
+      <c r="M3">
+        <v>0.25700000000000001</v>
+      </c>
+      <c r="N3">
         <v>-0.25</v>
       </c>
-      <c r="L2">
+      <c r="O3">
         <v>0.1</v>
       </c>
-      <c r="M2">
-        <v>0.5</v>
-      </c>
-      <c r="N2">
-        <v>0.2</v>
-      </c>
-      <c r="O2">
-        <v>0.5</v>
-      </c>
-      <c r="P2">
-        <v>4</v>
-      </c>
-      <c r="Q2">
+      <c r="P3">
+        <v>1</v>
+      </c>
+      <c r="Q3">
+        <v>1</v>
+      </c>
+      <c r="R3">
+        <v>0.6</v>
+      </c>
+      <c r="S3">
+        <v>0.5</v>
+      </c>
+      <c r="T3">
+        <v>13</v>
+      </c>
+      <c r="U3">
+        <v>2</v>
+      </c>
+      <c r="V3">
+        <v>0</v>
+      </c>
+      <c r="W3">
         <v>5</v>
       </c>
-      <c r="R2">
+      <c r="X3">
         <v>0.01</v>
       </c>
-      <c r="S2" s="3">
-        <v>1</v>
-      </c>
-      <c r="T2" s="3">
-        <v>20</v>
-      </c>
-      <c r="U2" s="3">
-        <v>10000000</v>
-      </c>
-      <c r="V2" s="3">
-        <v>0</v>
-      </c>
-      <c r="X2" t="s">
-        <v>45</v>
-      </c>
-      <c r="Y2" t="s">
-        <v>51</v>
-      </c>
-    </row>
-    <row r="3" spans="1:25" s="14" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="14" t="s">
+      <c r="Y3">
         <v>23</v>
       </c>
-      <c r="B3" s="14" t="s">
-        <v>2</v>
-      </c>
-      <c r="C3" s="14" t="s">
-        <v>33</v>
-      </c>
-      <c r="D3" s="14" t="s">
-        <v>15</v>
-      </c>
-      <c r="E3" s="14" t="s">
-        <v>43</v>
-      </c>
-      <c r="F3" s="14" t="s">
-        <v>16</v>
-      </c>
-      <c r="G3" s="14">
+      <c r="AA3">
+        <v>19</v>
+      </c>
+      <c r="AB3">
+        <v>59.5</v>
+      </c>
+      <c r="AC3">
+        <v>1000000000000000</v>
+      </c>
+      <c r="AD3">
         <v>1000</v>
       </c>
-      <c r="H3" s="14">
-        <v>1</v>
-      </c>
-      <c r="I3" s="14">
-        <v>1</v>
-      </c>
-      <c r="J3" s="14">
-        <v>0.25700000000000001</v>
-      </c>
-      <c r="K3" s="14">
-        <v>-0.25</v>
-      </c>
-      <c r="L3" s="14">
-        <v>0.1</v>
-      </c>
-      <c r="M3" s="14">
-        <v>1</v>
-      </c>
-      <c r="N3" s="14">
-        <v>0.6</v>
-      </c>
-      <c r="O3" s="14">
-        <v>0.5</v>
-      </c>
-      <c r="P3" s="14">
-        <v>13</v>
-      </c>
-      <c r="Q3" s="14">
-        <v>5</v>
-      </c>
-      <c r="R3" s="14">
-        <v>0.01</v>
-      </c>
-      <c r="S3" s="14">
-        <v>23</v>
-      </c>
-      <c r="T3" s="14">
-        <v>19</v>
-      </c>
-      <c r="U3" s="14">
-        <v>1000000000000000</v>
-      </c>
-      <c r="V3" s="14">
-        <v>1000</v>
-      </c>
-      <c r="X3" s="14" t="s">
-        <v>45</v>
-      </c>
-      <c r="Y3" s="14" t="s">
-        <v>57</v>
-      </c>
-    </row>
-    <row r="4" spans="1:25" s="3" customFormat="1" x14ac:dyDescent="0.3">
-      <c r="E4" s="14"/>
-      <c r="U4" s="14"/>
+      <c r="AF3" t="s">
+        <v>44</v>
+      </c>
+      <c r="AG3" t="s">
+        <v>56</v>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
@@ -1176,17 +1272,17 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{6C48BE33-A8B0-4574-8E5C-C0DC6671A66C}">
-  <dimension ref="A1:M1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:O1"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="16.44140625" customWidth="1"/>
-    <col min="5" max="6" width="24.44140625" customWidth="1"/>
-    <col min="7" max="7" width="22.33203125" customWidth="1"/>
-    <col min="8" max="8" width="16.88671875" customWidth="1"/>
-    <col min="11" max="12" width="15.44140625" customWidth="1"/>
+    <col min="1" max="1" width="16.42578125" customWidth="1"/>
+    <col min="5" max="6" width="24.42578125" customWidth="1"/>
+    <col min="7" max="8" width="22.28515625" customWidth="1"/>
+    <col min="9" max="9" width="16.85546875" customWidth="1"/>
+    <col min="12" max="14" width="15.42578125" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>6</v>
       </c>
@@ -1197,34 +1293,40 @@
         <v>1</v>
       </c>
       <c r="D1" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="E1" s="1" t="s">
         <v>39</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="F1" s="1" t="s">
         <v>40</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="G1" s="1" t="s">
         <v>41</v>
       </c>
-      <c r="G1" s="1" t="s">
-        <v>42</v>
-      </c>
       <c r="H1" s="1" t="s">
-        <v>24</v>
+        <v>70</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>46</v>
+        <v>23</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>28</v>
+        <v>45</v>
       </c>
       <c r="K1" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="L1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="L1" s="1" t="s">
-        <v>44</v>
-      </c>
       <c r="M1" s="1" t="s">
-        <v>38</v>
+        <v>5</v>
+      </c>
+      <c r="N1" s="1" t="s">
+        <v>43</v>
+      </c>
+      <c r="O1" s="1" t="s">
+        <v>37</v>
       </c>
     </row>
   </sheetData>
@@ -1235,2299 +1337,2298 @@
 <file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FF57B5C7-673A-4553-BCF4-7215DF8F4393}">
   <dimension ref="A1:D208"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="11.44140625" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="11.42578125" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="15.33203125" style="3" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="14.33203125" style="3" bestFit="1" customWidth="1"/>
-    <col min="3" max="16384" width="11.44140625" style="3"/>
+    <col min="1" max="1" width="15.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="14.28515625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A1" s="6" t="s">
+    <row r="1" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A1" s="5" t="s">
         <v>21</v>
       </c>
-      <c r="B1" s="7" t="s">
+      <c r="B1" s="6" t="s">
         <v>19</v>
       </c>
       <c r="C1" s="1" t="s">
-        <v>56</v>
-      </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A2" s="15">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="2" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A2" s="8">
         <v>44927.083333333336</v>
       </c>
-      <c r="B2" s="4">
+      <c r="B2" s="3">
         <v>1.2824365603285201E-4</v>
       </c>
-      <c r="C2" s="5">
+      <c r="C2" s="4">
         <v>0.1</v>
       </c>
       <c r="D2" s="2"/>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A3" s="15">
+    <row r="3" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A3" s="8">
         <v>44927.125</v>
       </c>
-      <c r="B3" s="4">
+      <c r="B3" s="3">
         <v>1.3149033086912699E-4</v>
       </c>
-      <c r="C3" s="5">
+      <c r="C3" s="4">
         <v>0.2</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A4" s="15">
+    <row r="4" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A4" s="8">
         <v>44927.166666666664</v>
       </c>
-      <c r="B4" s="4">
+      <c r="B4" s="3">
         <v>1.417714678506636E-4</v>
       </c>
-      <c r="C4" s="5">
+      <c r="C4" s="4">
         <v>0.3</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A5" s="15">
+    <row r="5" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A5" s="8">
         <v>44927.208333333336</v>
       </c>
-      <c r="B5" s="4">
+      <c r="B5" s="3">
         <v>1.6882709148628681E-4</v>
       </c>
-      <c r="C5" s="5">
+      <c r="C5" s="4">
         <v>0.4</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A6" s="15">
+    <row r="6" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A6" s="8">
         <v>44927.25</v>
       </c>
-      <c r="B6" s="4">
+      <c r="B6" s="3">
         <v>2.4241838777518099E-4</v>
       </c>
-      <c r="C6" s="5">
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A7" s="15">
+      <c r="C6" s="4">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="7" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A7" s="8">
         <v>44927.291666666664</v>
       </c>
-      <c r="B7" s="4">
+      <c r="B7" s="3">
         <v>3.1222189675508762E-4</v>
       </c>
-      <c r="C7" s="5">
+      <c r="C7" s="4">
         <v>0.6</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A8" s="15">
+    <row r="8" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A8" s="8">
         <v>44927.333333333336</v>
       </c>
-      <c r="B8" s="4">
+      <c r="B8" s="3">
         <v>2.9057739784658942E-4</v>
       </c>
-      <c r="C8" s="5">
+      <c r="C8" s="4">
         <v>0.7</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A9" s="15">
+    <row r="9" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A9" s="8">
         <v>44927.375</v>
       </c>
-      <c r="B9" s="4">
+      <c r="B9" s="3">
         <v>2.7596736108335279E-4</v>
       </c>
-      <c r="C9" s="5">
+      <c r="C9" s="4">
         <v>0.6</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A10" s="15">
+    <row r="10" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A10" s="8">
         <v>44927.416666666664</v>
       </c>
-      <c r="B10" s="4">
+      <c r="B10" s="3">
         <v>2.6406288668367897E-4</v>
       </c>
-      <c r="C10" s="5">
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="11" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A11" s="15">
+      <c r="C10" s="4">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="11" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A11" s="8">
         <v>44927.458333333336</v>
       </c>
-      <c r="B11" s="4">
+      <c r="B11" s="3">
         <v>2.5161729981129199E-4</v>
       </c>
-      <c r="C11" s="5">
+      <c r="C11" s="4">
         <v>0.4</v>
       </c>
     </row>
-    <row r="12" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A12" s="15">
+    <row r="12" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A12" s="8">
         <v>44927.5</v>
       </c>
-      <c r="B12" s="4">
+      <c r="B12" s="3">
         <v>2.4241838777518099E-4</v>
       </c>
-      <c r="C12" s="5">
+      <c r="C12" s="4">
         <v>0.3</v>
       </c>
     </row>
-    <row r="13" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A13" s="15">
+    <row r="13" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A13" s="8">
         <v>44927.541666666664</v>
       </c>
-      <c r="B13" s="4">
+      <c r="B13" s="3">
         <v>2.3700726304805601E-4</v>
       </c>
-      <c r="C13" s="5">
+      <c r="C13" s="4">
         <v>0.2</v>
       </c>
     </row>
-    <row r="14" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A14" s="15">
+    <row r="14" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A14" s="8">
         <v>44927.583333333336</v>
       </c>
-      <c r="B14" s="4">
+      <c r="B14" s="3">
         <v>2.36466150575344E-4</v>
       </c>
-      <c r="C14" s="5">
+      <c r="C14" s="4">
         <v>0.1</v>
       </c>
     </row>
-    <row r="15" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A15" s="15">
+    <row r="15" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A15" s="8">
         <v>44927.625</v>
       </c>
-      <c r="B15" s="4">
+      <c r="B15" s="3">
         <v>2.4133616282975579E-4</v>
       </c>
-      <c r="C15" s="5">
+      <c r="C15" s="4">
         <v>0.2</v>
       </c>
     </row>
-    <row r="16" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A16" s="15">
+    <row r="16" spans="1:4" x14ac:dyDescent="0.25">
+      <c r="A16" s="8">
         <v>44927.666666666664</v>
       </c>
-      <c r="B16" s="4">
+      <c r="B16" s="3">
         <v>2.47829512502305E-4</v>
       </c>
-      <c r="C16" s="5">
+      <c r="C16" s="4">
         <v>0.3</v>
       </c>
     </row>
-    <row r="17" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A17" s="15">
+    <row r="17" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A17" s="8">
         <v>44927.708333333336</v>
       </c>
-      <c r="B17" s="4">
+      <c r="B17" s="3">
         <v>2.6027509937469182E-4</v>
       </c>
-      <c r="C17" s="5">
+      <c r="C17" s="4">
         <v>0.4</v>
       </c>
     </row>
-    <row r="18" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A18" s="15">
+    <row r="18" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A18" s="8">
         <v>44927.75</v>
       </c>
-      <c r="B18" s="4">
+      <c r="B18" s="3">
         <v>2.710973488289406E-4</v>
       </c>
-      <c r="C18" s="5">
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="19" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A19" s="15">
+      <c r="C18" s="4">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A19" s="8">
         <v>44927.791666666664</v>
       </c>
-      <c r="B19" s="4">
+      <c r="B19" s="3">
         <v>2.7380291119250341E-4</v>
       </c>
-      <c r="C19" s="5">
+      <c r="C19" s="4">
         <v>0.6</v>
       </c>
     </row>
-    <row r="20" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A20" s="15">
+    <row r="20" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A20" s="8">
         <v>44927.833333333336</v>
       </c>
-      <c r="B20" s="4">
+      <c r="B20" s="3">
         <v>2.7326179871979062E-4</v>
       </c>
-      <c r="C20" s="5">
+      <c r="C20" s="4">
         <v>0.7</v>
       </c>
     </row>
-    <row r="21" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A21" s="15">
+    <row r="21" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A21" s="8">
         <v>44927.875</v>
       </c>
-      <c r="B21" s="4">
+      <c r="B21" s="3">
         <v>2.6243954926554179E-4</v>
       </c>
-      <c r="C21" s="5">
+      <c r="C21" s="4">
         <v>0.6</v>
       </c>
     </row>
-    <row r="22" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A22" s="15">
+    <row r="22" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A22" s="8">
         <v>44927.916666666664</v>
       </c>
-      <c r="B22" s="4">
+      <c r="B22" s="3">
         <v>2.3267836326635639E-4</v>
       </c>
-      <c r="C22" s="5">
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="23" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A23" s="15">
+      <c r="C22" s="4">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="23" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A23" s="8">
         <v>44927.958333333336</v>
       </c>
-      <c r="B23" s="4">
+      <c r="B23" s="3">
         <v>1.6720375406814901E-4</v>
       </c>
-      <c r="C23" s="5">
+      <c r="C23" s="4">
         <v>0.4</v>
       </c>
     </row>
-    <row r="24" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A24" s="15">
+    <row r="24" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A24" s="8">
         <v>44928</v>
       </c>
-      <c r="B24" s="4">
+      <c r="B24" s="3">
         <v>1.331136682872642E-4</v>
       </c>
-      <c r="C24" s="5">
+      <c r="C24" s="4">
         <v>0.3</v>
       </c>
     </row>
-    <row r="25" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A25" s="15">
+    <row r="25" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A25" s="8">
         <v>44928.041666666664</v>
       </c>
-      <c r="B25" s="4">
+      <c r="B25" s="3">
         <v>1.1112192823917541E-4</v>
       </c>
-      <c r="C25" s="5">
+      <c r="C25" s="4">
         <v>0.2</v>
       </c>
     </row>
-    <row r="26" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A26" s="15">
+    <row r="26" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A26" s="8">
         <v>44928.083333333336</v>
       </c>
-      <c r="B26" s="4">
+      <c r="B26" s="3">
         <v>1.145038999681938E-4</v>
       </c>
-      <c r="C26" s="5">
+      <c r="C26" s="4">
         <v>0.1</v>
       </c>
     </row>
-    <row r="27" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A27" s="15">
+    <row r="27" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A27" s="8">
         <v>44928.125</v>
       </c>
-      <c r="B27" s="4">
+      <c r="B27" s="3">
         <v>1.17402732878781E-4</v>
       </c>
-      <c r="C27" s="5">
+      <c r="C27" s="4">
         <v>0.2</v>
       </c>
     </row>
-    <row r="28" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A28" s="15">
+    <row r="28" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A28" s="8">
         <v>44928.166666666664</v>
       </c>
-      <c r="B28" s="4">
+      <c r="B28" s="3">
         <v>1.2658237042897379E-4</v>
       </c>
-      <c r="C28" s="5">
+      <c r="C28" s="4">
         <v>0.3</v>
       </c>
     </row>
-    <row r="29" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A29" s="15">
+    <row r="29" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A29" s="8">
         <v>44928.208333333336</v>
       </c>
-      <c r="B29" s="4">
+      <c r="B29" s="3">
         <v>1.5073931135053381E-4</v>
       </c>
-      <c r="C29" s="5">
+      <c r="C29" s="4">
         <v>0.4</v>
       </c>
     </row>
-    <row r="30" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A30" s="15">
+    <row r="30" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A30" s="8">
         <v>44928.25</v>
       </c>
-      <c r="B30" s="4">
+      <c r="B30" s="3">
         <v>2.16446190657177E-4</v>
       </c>
-      <c r="C30" s="5">
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="31" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A31" s="15">
+      <c r="C30" s="4">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="31" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A31" s="8">
         <v>44928.291666666664</v>
       </c>
-      <c r="B31" s="4">
+      <c r="B31" s="3">
         <v>2.7877109823480118E-4</v>
       </c>
-      <c r="C31" s="5">
+      <c r="C31" s="4">
         <v>0.6</v>
       </c>
     </row>
-    <row r="32" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A32" s="15">
+    <row r="32" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A32" s="8">
         <v>44928.333333333336</v>
       </c>
-      <c r="B32" s="4">
+      <c r="B32" s="3">
         <v>2.5944554549755302E-4</v>
       </c>
-      <c r="C32" s="5">
+      <c r="C32" s="4">
         <v>0.7</v>
       </c>
     </row>
-    <row r="33" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A33" s="15">
+    <row r="33" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A33" s="8">
         <v>44928.375</v>
       </c>
-      <c r="B33" s="4">
+      <c r="B33" s="3">
         <v>2.4640079739991078E-4</v>
       </c>
-      <c r="C33" s="5">
+      <c r="C33" s="4">
         <v>0.6</v>
       </c>
     </row>
-    <row r="34" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A34" s="15">
+    <row r="34" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A34" s="8">
         <v>44928.416666666664</v>
       </c>
-      <c r="B34" s="4">
+      <c r="B34" s="3">
         <v>2.357717433944244E-4</v>
       </c>
-      <c r="C34" s="5">
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="35" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A35" s="15">
+      <c r="C34" s="4">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="35" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A35" s="8">
         <v>44928.458333333336</v>
       </c>
-      <c r="B35" s="4">
+      <c r="B35" s="3">
         <v>2.2465955057050679E-4</v>
       </c>
-      <c r="C35" s="5">
+      <c r="C35" s="4">
         <v>0.4</v>
       </c>
     </row>
-    <row r="36" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A36" s="15">
+    <row r="36" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A36" s="8">
         <v>44928.5</v>
       </c>
-      <c r="B36" s="4">
+      <c r="B36" s="3">
         <v>2.16446190657177E-4</v>
       </c>
-      <c r="C36" s="5">
+      <c r="C36" s="4">
         <v>0.3</v>
       </c>
     </row>
-    <row r="37" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A37" s="15">
+    <row r="37" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A37" s="8">
         <v>44928.541666666664</v>
       </c>
-      <c r="B37" s="4">
+      <c r="B37" s="3">
         <v>2.1161480247286501E-4</v>
       </c>
-      <c r="C37" s="5">
+      <c r="C37" s="4">
         <v>0.2</v>
       </c>
     </row>
-    <row r="38" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A38" s="15">
+    <row r="38" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A38" s="8">
         <v>44928.583333333336</v>
       </c>
-      <c r="B38" s="4">
+      <c r="B38" s="3">
         <v>2.111316636544338E-4</v>
       </c>
-      <c r="C38" s="5">
+      <c r="C38" s="4">
         <v>0.1</v>
       </c>
     </row>
-    <row r="39" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A39" s="15">
+    <row r="39" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A39" s="8">
         <v>44928.625</v>
       </c>
-      <c r="B39" s="4">
+      <c r="B39" s="3">
         <v>2.154799130203146E-4</v>
       </c>
-      <c r="C39" s="5">
+      <c r="C39" s="4">
         <v>0.2</v>
       </c>
     </row>
-    <row r="40" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A40" s="15">
+    <row r="40" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A40" s="8">
         <v>44928.666666666664</v>
       </c>
-      <c r="B40" s="4">
+      <c r="B40" s="3">
         <v>2.2127757884148901E-4</v>
       </c>
-      <c r="C40" s="5">
+      <c r="C40" s="4">
         <v>0.3</v>
       </c>
     </row>
-    <row r="41" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A41" s="15">
+    <row r="41" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A41" s="8">
         <v>44928.708333333336</v>
       </c>
-      <c r="B41" s="4">
+      <c r="B41" s="3">
         <v>2.32389771665406E-4</v>
       </c>
-      <c r="C41" s="5">
+      <c r="C41" s="4">
         <v>0.4</v>
       </c>
     </row>
-    <row r="42" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A42" s="15">
+    <row r="42" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A42" s="8">
         <v>44928.75</v>
       </c>
-      <c r="B42" s="4">
+      <c r="B42" s="3">
         <v>2.4205254803403E-4</v>
       </c>
-      <c r="C42" s="5">
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="43" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A43" s="15">
+      <c r="C42" s="4">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="43" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A43" s="8">
         <v>44928.791666666664</v>
       </c>
-      <c r="B43" s="4">
+      <c r="B43" s="3">
         <v>2.4446824212618598E-4</v>
       </c>
-      <c r="C43" s="5">
+      <c r="C43" s="4">
         <v>0.6</v>
       </c>
     </row>
-    <row r="44" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A44" s="15">
+    <row r="44" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A44" s="8">
         <v>44928.833333333336</v>
       </c>
-      <c r="B44" s="4">
+      <c r="B44" s="3">
         <v>2.439851033077548E-4</v>
       </c>
-      <c r="C44" s="5">
+      <c r="C44" s="4">
         <v>0.7</v>
       </c>
     </row>
-    <row r="45" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A45" s="15">
+    <row r="45" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A45" s="8">
         <v>44928.875</v>
       </c>
-      <c r="B45" s="4">
+      <c r="B45" s="3">
         <v>2.3432232693913101E-4</v>
       </c>
-      <c r="C45" s="5">
+      <c r="C45" s="4">
         <v>0.6</v>
       </c>
     </row>
-    <row r="46" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A46" s="15">
+    <row r="46" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A46" s="8">
         <v>44928.916666666664</v>
       </c>
-      <c r="B46" s="4">
+      <c r="B46" s="3">
         <v>2.0774969192541539E-4</v>
       </c>
-      <c r="C46" s="5">
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="47" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A47" s="15">
+      <c r="C46" s="4">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="47" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A47" s="8">
         <v>44928.958333333336</v>
       </c>
-      <c r="B47" s="4">
+      <c r="B47" s="3">
         <v>1.492898948952402E-4</v>
       </c>
-      <c r="C47" s="5">
+      <c r="C47" s="4">
         <v>0.4</v>
       </c>
     </row>
-    <row r="48" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A48" s="15">
+    <row r="48" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A48" s="8">
         <v>44929</v>
       </c>
-      <c r="B48" s="4">
+      <c r="B48" s="3">
         <v>1.1885214933407501E-4</v>
       </c>
-      <c r="C48" s="5">
+      <c r="C48" s="4">
         <v>0.3</v>
       </c>
     </row>
-    <row r="49" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A49" s="15">
+    <row r="49" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A49" s="8">
         <v>44929.041666666664</v>
       </c>
-      <c r="B49" s="4">
+      <c r="B49" s="3">
         <v>1.17821643065071E-4</v>
       </c>
-      <c r="C49" s="5">
+      <c r="C49" s="4">
         <v>0.2</v>
       </c>
     </row>
-    <row r="50" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A50" s="15">
+    <row r="50" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A50" s="8">
         <v>44929.083333333336</v>
       </c>
-      <c r="B50" s="4">
+      <c r="B50" s="3">
         <v>1.21407519158355E-4</v>
       </c>
-      <c r="C50" s="5">
+      <c r="C50" s="4">
         <v>0.1</v>
       </c>
     </row>
-    <row r="51" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A51" s="15">
+    <row r="51" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A51" s="8">
         <v>44929.125</v>
       </c>
-      <c r="B51" s="4">
+      <c r="B51" s="3">
         <v>1.2448112723831341E-4</v>
       </c>
-      <c r="C51" s="5">
+      <c r="C51" s="4">
         <v>0.2</v>
       </c>
     </row>
-    <row r="52" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A52" s="15">
+    <row r="52" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A52" s="8">
         <v>44929.166666666664</v>
       </c>
-      <c r="B52" s="4">
+      <c r="B52" s="3">
         <v>1.342142194915152E-4</v>
       </c>
-      <c r="C52" s="5">
+      <c r="C52" s="4">
         <v>0.3</v>
       </c>
     </row>
-    <row r="53" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A53" s="15">
+    <row r="53" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A53" s="8">
         <v>44929.208333333336</v>
       </c>
-      <c r="B53" s="4">
+      <c r="B53" s="3">
         <v>1.598276201578344E-4</v>
       </c>
-      <c r="C53" s="5">
+      <c r="C53" s="4">
         <v>0.4</v>
       </c>
     </row>
-    <row r="54" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A54" s="15">
+    <row r="54" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A54" s="8">
         <v>44929.25</v>
       </c>
-      <c r="B54" s="4">
+      <c r="B54" s="3">
         <v>2.294960699702244E-4</v>
       </c>
-      <c r="C54" s="5">
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="55" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A55" s="15">
+      <c r="C54" s="4">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="55" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A55" s="8">
         <v>44929.291666666664</v>
       </c>
-      <c r="B55" s="4">
+      <c r="B55" s="3">
         <v>2.9557864368932879E-4</v>
       </c>
-      <c r="C55" s="5">
+      <c r="C55" s="4">
         <v>0.6</v>
       </c>
     </row>
-    <row r="56" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A56" s="15">
+    <row r="56" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A56" s="8">
         <v>44929.333333333336</v>
       </c>
-      <c r="B56" s="4">
+      <c r="B56" s="3">
         <v>2.7508792315627319E-4</v>
       </c>
-      <c r="C56" s="5">
+      <c r="C56" s="4">
         <v>0.7</v>
       </c>
     </row>
-    <row r="57" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A57" s="15">
+    <row r="57" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A57" s="8">
         <v>44929.375</v>
       </c>
-      <c r="B57" s="4">
+      <c r="B57" s="3">
         <v>2.6125668679646038E-4</v>
       </c>
-      <c r="C57" s="5">
+      <c r="C57" s="4">
         <v>0.6</v>
       </c>
     </row>
-    <row r="58" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A58" s="15">
+    <row r="58" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A58" s="8">
         <v>44929.416666666664</v>
       </c>
-      <c r="B58" s="4">
+      <c r="B58" s="3">
         <v>2.4998679050328002E-4</v>
       </c>
-      <c r="C58" s="5">
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="59" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A59" s="15">
+      <c r="C58" s="4">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="59" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A59" s="8">
         <v>44929.458333333336</v>
       </c>
-      <c r="B59" s="4">
+      <c r="B59" s="3">
         <v>2.3820462619677301E-4</v>
       </c>
-      <c r="C59" s="5">
+      <c r="C59" s="4">
         <v>0.4</v>
       </c>
     </row>
-    <row r="60" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A60" s="15">
+    <row r="60" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A60" s="8">
         <v>44929.5</v>
       </c>
-      <c r="B60" s="4">
+      <c r="B60" s="3">
         <v>2.294960699702244E-4</v>
       </c>
-      <c r="C60" s="5">
+      <c r="C60" s="4">
         <v>0.3</v>
       </c>
     </row>
-    <row r="61" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A61" s="15">
+    <row r="61" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A61" s="8">
         <v>44929.541666666664</v>
       </c>
-      <c r="B61" s="4">
+      <c r="B61" s="3">
         <v>2.243733898369602E-4</v>
       </c>
-      <c r="C61" s="5">
+      <c r="C61" s="4">
         <v>0.2</v>
       </c>
     </row>
-    <row r="62" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A62" s="15">
+    <row r="62" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A62" s="8">
         <v>44929.583333333336</v>
       </c>
-      <c r="B62" s="4">
+      <c r="B62" s="3">
         <v>2.23861121823634E-4</v>
       </c>
-      <c r="C62" s="5">
+      <c r="C62" s="4">
         <v>0.1</v>
       </c>
     </row>
-    <row r="63" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A63" s="15">
+    <row r="63" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A63" s="8">
         <v>44929.625</v>
       </c>
-      <c r="B63" s="4">
+      <c r="B63" s="3">
         <v>2.2847153394357119E-4</v>
       </c>
-      <c r="C63" s="5">
+      <c r="C63" s="4">
         <v>0.2</v>
       </c>
     </row>
-    <row r="64" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A64" s="15">
+    <row r="64" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A64" s="8">
         <v>44929.666666666664</v>
       </c>
-      <c r="B64" s="4">
+      <c r="B64" s="3">
         <v>2.34618750103488E-4</v>
       </c>
-      <c r="C64" s="5">
+      <c r="C64" s="4">
         <v>0.3</v>
       </c>
     </row>
-    <row r="65" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A65" s="15">
+    <row r="65" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A65" s="8">
         <v>44929.708333333336</v>
       </c>
-      <c r="B65" s="4">
+      <c r="B65" s="3">
         <v>2.4640091440999501E-4</v>
       </c>
-      <c r="C65" s="5">
+      <c r="C65" s="4">
         <v>0.4</v>
       </c>
     </row>
-    <row r="66" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A66" s="15">
+    <row r="66" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A66" s="8">
         <v>44929.75</v>
       </c>
-      <c r="B66" s="4">
+      <c r="B66" s="3">
         <v>2.5664627467652298E-4</v>
       </c>
-      <c r="C66" s="5">
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="67" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A67" s="15">
+      <c r="C66" s="4">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="67" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A67" s="8">
         <v>44929.791666666664</v>
       </c>
-      <c r="B67" s="4">
+      <c r="B67" s="3">
         <v>2.5920761474315499E-4</v>
       </c>
-      <c r="C67" s="5">
+      <c r="C67" s="4">
         <v>0.6</v>
       </c>
     </row>
-    <row r="68" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A68" s="15">
+    <row r="68" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A68" s="8">
         <v>44929.833333333336</v>
       </c>
-      <c r="B68" s="4">
+      <c r="B68" s="3">
         <v>2.5869534672982858E-4</v>
       </c>
-      <c r="C68" s="5">
+      <c r="C68" s="4">
         <v>0.7</v>
       </c>
     </row>
-    <row r="69" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A69" s="15">
+    <row r="69" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A69" s="8">
         <v>44929.875</v>
       </c>
-      <c r="B69" s="4">
+      <c r="B69" s="3">
         <v>2.4844998646330078E-4</v>
       </c>
-      <c r="C69" s="5">
+      <c r="C69" s="4">
         <v>0.6</v>
       </c>
     </row>
-    <row r="70" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A70" s="15">
+    <row r="70" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A70" s="8">
         <v>44929.916666666664</v>
       </c>
-      <c r="B70" s="4">
+      <c r="B70" s="3">
         <v>2.2027524573034921E-4</v>
       </c>
-      <c r="C70" s="5">
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="71" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A71" s="15">
+      <c r="C70" s="4">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="71" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A71" s="8">
         <v>44929.958333333336</v>
       </c>
-      <c r="B71" s="4">
+      <c r="B71" s="3">
         <v>1.5829081611785521E-4</v>
       </c>
-      <c r="C71" s="5">
+      <c r="C71" s="4">
         <v>0.4</v>
       </c>
     </row>
-    <row r="72" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A72" s="15">
+    <row r="72" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A72" s="8">
         <v>44930</v>
       </c>
-      <c r="B72" s="4">
+      <c r="B72" s="3">
         <v>1.260179312782926E-4</v>
       </c>
-      <c r="C72" s="5">
+      <c r="C72" s="4">
         <v>0.3</v>
       </c>
     </row>
-    <row r="73" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A73" s="15">
+    <row r="73" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A73" s="8">
         <v>44930.041666666664</v>
       </c>
-      <c r="B73" s="4">
+      <c r="B73" s="3">
         <v>1.265761578251604E-4</v>
       </c>
-      <c r="C73" s="5">
+      <c r="C73" s="4">
         <v>0.2</v>
       </c>
     </row>
-    <row r="74" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A74" s="15">
+    <row r="74" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A74" s="8">
         <v>44930.083333333336</v>
       </c>
-      <c r="B74" s="4">
+      <c r="B74" s="3">
         <v>1.304284756720128E-4</v>
       </c>
-      <c r="C74" s="5">
+      <c r="C74" s="4">
         <v>0.1</v>
       </c>
     </row>
-    <row r="75" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A75" s="15">
+    <row r="75" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A75" s="8">
         <v>44930.125</v>
       </c>
-      <c r="B75" s="4">
+      <c r="B75" s="3">
         <v>1.33730462397887E-4</v>
       </c>
-      <c r="C75" s="5">
+      <c r="C75" s="4">
         <v>0.2</v>
       </c>
     </row>
-    <row r="76" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A76" s="15">
+    <row r="76" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A76" s="8">
         <v>44930.166666666664</v>
       </c>
-      <c r="B76" s="4">
+      <c r="B76" s="3">
         <v>1.441867536964872E-4</v>
       </c>
-      <c r="C76" s="5">
+      <c r="C76" s="4">
         <v>0.3</v>
       </c>
     </row>
-    <row r="77" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A77" s="15">
+    <row r="77" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A77" s="8">
         <v>44930.208333333336</v>
       </c>
-      <c r="B77" s="4">
+      <c r="B77" s="3">
         <v>1.7170330974543481E-4</v>
       </c>
-      <c r="C77" s="5">
+      <c r="C77" s="4">
         <v>0.4</v>
       </c>
     </row>
-    <row r="78" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A78" s="15">
+    <row r="78" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A78" s="8">
         <v>44930.25</v>
       </c>
-      <c r="B78" s="4">
+      <c r="B78" s="3">
         <v>2.46548342198573E-4</v>
       </c>
-      <c r="C78" s="5">
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="79" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A79" s="15">
+      <c r="C78" s="4">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="79" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A79" s="8">
         <v>44930.291666666664</v>
       </c>
-      <c r="B79" s="4">
+      <c r="B79" s="3">
         <v>3.1754105680485798E-4</v>
       </c>
-      <c r="C79" s="5">
+      <c r="C79" s="4">
         <v>0.6</v>
       </c>
     </row>
-    <row r="80" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A80" s="15">
+    <row r="80" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A80" s="8">
         <v>44930.333333333336</v>
       </c>
-      <c r="B80" s="4">
+      <c r="B80" s="3">
         <v>2.9552781196570021E-4</v>
       </c>
-      <c r="C80" s="5">
+      <c r="C80" s="4">
         <v>0.7</v>
       </c>
     </row>
-    <row r="81" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A81" s="15">
+    <row r="81" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A81" s="8">
         <v>44930.375</v>
       </c>
-      <c r="B81" s="4">
+      <c r="B81" s="3">
         <v>2.8066887169926841E-4</v>
       </c>
-      <c r="C81" s="5">
+      <c r="C81" s="4">
         <v>0.6</v>
       </c>
     </row>
-    <row r="82" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A82" s="15">
+    <row r="82" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A82" s="8">
         <v>44930.416666666664</v>
       </c>
-      <c r="B82" s="4">
+      <c r="B82" s="3">
         <v>2.6856158703773202E-4</v>
       </c>
-      <c r="C82" s="5">
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="83" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A83" s="15">
+      <c r="C82" s="4">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="83" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A83" s="8">
         <v>44930.458333333336</v>
       </c>
-      <c r="B83" s="4">
+      <c r="B83" s="3">
         <v>2.5590397125521518E-4</v>
       </c>
-      <c r="C83" s="5">
+      <c r="C83" s="4">
         <v>0.4</v>
       </c>
     </row>
-    <row r="84" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A84" s="15">
+    <row r="84" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A84" s="8">
         <v>44930.5</v>
       </c>
-      <c r="B84" s="4">
+      <c r="B84" s="3">
         <v>2.46548342198573E-4</v>
       </c>
-      <c r="C84" s="5">
+      <c r="C84" s="4">
         <v>0.3</v>
       </c>
     </row>
-    <row r="85" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A85" s="15">
+    <row r="85" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A85" s="8">
         <v>44930.541666666664</v>
       </c>
-      <c r="B85" s="4">
+      <c r="B85" s="3">
         <v>2.4104503098878341E-4</v>
       </c>
-      <c r="C85" s="5">
+      <c r="C85" s="4">
         <v>0.2</v>
       </c>
     </row>
-    <row r="86" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A86" s="15">
+    <row r="86" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A86" s="8">
         <v>44930.583333333336</v>
       </c>
-      <c r="B86" s="4">
+      <c r="B86" s="3">
         <v>2.4049469986780439E-4</v>
       </c>
-      <c r="C86" s="5">
+      <c r="C86" s="4">
         <v>0.1</v>
       </c>
     </row>
-    <row r="87" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A87" s="15">
+    <row r="87" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A87" s="8">
         <v>44930.625</v>
       </c>
-      <c r="B87" s="4">
+      <c r="B87" s="3">
         <v>2.4544767995661498E-4</v>
       </c>
-      <c r="C87" s="5">
+      <c r="C87" s="4">
         <v>0.2</v>
       </c>
     </row>
-    <row r="88" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A88" s="15">
+    <row r="88" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A88" s="8">
         <v>44930.666666666664</v>
       </c>
-      <c r="B88" s="4">
+      <c r="B88" s="3">
         <v>2.52051653408363E-4</v>
       </c>
-      <c r="C88" s="5">
+      <c r="C88" s="4">
         <v>0.3</v>
       </c>
     </row>
-    <row r="89" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A89" s="15">
+    <row r="89" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A89" s="8">
         <v>44930.708333333336</v>
       </c>
-      <c r="B89" s="4">
+      <c r="B89" s="3">
         <v>2.6470926919087859E-4</v>
       </c>
-      <c r="C89" s="5">
+      <c r="C89" s="4">
         <v>0.4</v>
       </c>
     </row>
-    <row r="90" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A90" s="15">
+    <row r="90" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A90" s="8">
         <v>44930.75</v>
       </c>
-      <c r="B90" s="4">
+      <c r="B90" s="3">
         <v>2.7571589161045799E-4</v>
       </c>
-      <c r="C90" s="5">
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="91" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A91" s="15">
+      <c r="C90" s="4">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="91" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A91" s="8">
         <v>44930.791666666664</v>
       </c>
-      <c r="B91" s="4">
+      <c r="B91" s="3">
         <v>2.7846754721535199E-4</v>
       </c>
-      <c r="C91" s="5">
+      <c r="C91" s="4">
         <v>0.6</v>
       </c>
     </row>
-    <row r="92" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A92" s="15">
+    <row r="92" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A92" s="8">
         <v>44930.833333333336</v>
       </c>
-      <c r="B92" s="4">
+      <c r="B92" s="3">
         <v>2.77917216094373E-4</v>
       </c>
-      <c r="C92" s="5">
+      <c r="C92" s="4">
         <v>0.7</v>
       </c>
     </row>
-    <row r="93" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A93" s="15">
+    <row r="93" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A93" s="8">
         <v>44930.875</v>
       </c>
-      <c r="B93" s="4">
+      <c r="B93" s="3">
         <v>2.6691059367479458E-4</v>
       </c>
-      <c r="C93" s="5">
+      <c r="C93" s="4">
         <v>0.6</v>
       </c>
     </row>
-    <row r="94" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A94" s="15">
+    <row r="94" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A94" s="8">
         <v>44930.916666666664</v>
       </c>
-      <c r="B94" s="4">
+      <c r="B94" s="3">
         <v>2.36642382020952E-4</v>
       </c>
-      <c r="C94" s="5">
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="95" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A95" s="15">
+      <c r="C94" s="4">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="95" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A95" s="8">
         <v>44930.958333333336</v>
       </c>
-      <c r="B95" s="4">
+      <c r="B95" s="3">
         <v>1.700523163824978E-4</v>
       </c>
-      <c r="C95" s="5">
+      <c r="C95" s="4">
         <v>0.4</v>
       </c>
     </row>
-    <row r="96" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A96" s="15">
+    <row r="96" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A96" s="8">
         <v>44931</v>
       </c>
-      <c r="B96" s="4">
+      <c r="B96" s="3">
         <v>1.331136682872642E-4</v>
       </c>
-      <c r="C96" s="5">
+      <c r="C96" s="4">
         <v>0.3</v>
       </c>
     </row>
-    <row r="97" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A97" s="15">
+    <row r="97" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A97" s="8">
         <v>44931.041666666664</v>
       </c>
-      <c r="B97" s="4">
+      <c r="B97" s="3">
         <v>1.1112192823917541E-4</v>
       </c>
-      <c r="C97" s="5">
+      <c r="C97" s="4">
         <v>0.2</v>
       </c>
     </row>
-    <row r="98" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A98" s="15">
+    <row r="98" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A98" s="8">
         <v>44931.083333333336</v>
       </c>
-      <c r="B98" s="4">
+      <c r="B98" s="3">
         <v>1.145038999681938E-4</v>
       </c>
-      <c r="C98" s="5">
+      <c r="C98" s="4">
         <v>0.1</v>
       </c>
     </row>
-    <row r="99" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A99" s="15">
+    <row r="99" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A99" s="8">
         <v>44931.125</v>
       </c>
-      <c r="B99" s="4">
+      <c r="B99" s="3">
         <v>1.17402732878781E-4</v>
       </c>
-      <c r="C99" s="5">
+      <c r="C99" s="4">
         <v>0.2</v>
       </c>
     </row>
-    <row r="100" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A100" s="15">
+    <row r="100" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A100" s="8">
         <v>44931.166666666664</v>
       </c>
-      <c r="B100" s="4">
+      <c r="B100" s="3">
         <v>1.2658237042897379E-4</v>
       </c>
-      <c r="C100" s="5">
+      <c r="C100" s="4">
         <v>0.3</v>
       </c>
     </row>
-    <row r="101" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A101" s="15">
+    <row r="101" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A101" s="8">
         <v>44931.208333333336</v>
       </c>
-      <c r="B101" s="4">
+      <c r="B101" s="3">
         <v>1.5073931135053381E-4</v>
       </c>
-      <c r="C101" s="5">
+      <c r="C101" s="4">
         <v>0.4</v>
       </c>
     </row>
-    <row r="102" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A102" s="15">
+    <row r="102" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A102" s="8">
         <v>44931.25</v>
       </c>
-      <c r="B102" s="4">
+      <c r="B102" s="3">
         <v>2.16446190657177E-4</v>
       </c>
-      <c r="C102" s="5">
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="103" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A103" s="15">
+      <c r="C102" s="4">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="103" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A103" s="8">
         <v>44931.291666666664</v>
       </c>
-      <c r="B103" s="4">
+      <c r="B103" s="3">
         <v>2.7877109823480118E-4</v>
       </c>
-      <c r="C103" s="5">
+      <c r="C103" s="4">
         <v>0.6</v>
       </c>
     </row>
-    <row r="104" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A104" s="15">
+    <row r="104" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A104" s="8">
         <v>44931.333333333336</v>
       </c>
-      <c r="B104" s="4">
+      <c r="B104" s="3">
         <v>2.5944554549755302E-4</v>
       </c>
-      <c r="C104" s="5">
+      <c r="C104" s="4">
         <v>0.7</v>
       </c>
     </row>
-    <row r="105" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A105" s="15">
+    <row r="105" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A105" s="8">
         <v>44931.375</v>
       </c>
-      <c r="B105" s="4">
+      <c r="B105" s="3">
         <v>2.4640079739991078E-4</v>
       </c>
-      <c r="C105" s="5">
+      <c r="C105" s="4">
         <v>0.6</v>
       </c>
     </row>
-    <row r="106" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A106" s="15">
+    <row r="106" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A106" s="8">
         <v>44931.416666666664</v>
       </c>
-      <c r="B106" s="4">
+      <c r="B106" s="3">
         <v>2.357717433944244E-4</v>
       </c>
-      <c r="C106" s="5">
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="107" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A107" s="15">
+      <c r="C106" s="4">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="107" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A107" s="8">
         <v>44931.458333333336</v>
       </c>
-      <c r="B107" s="4">
+      <c r="B107" s="3">
         <v>2.2465955057050679E-4</v>
       </c>
-      <c r="C107" s="5">
+      <c r="C107" s="4">
         <v>0.4</v>
       </c>
     </row>
-    <row r="108" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A108" s="15">
+    <row r="108" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A108" s="8">
         <v>44931.5</v>
       </c>
-      <c r="B108" s="4">
+      <c r="B108" s="3">
         <v>2.16446190657177E-4</v>
       </c>
-      <c r="C108" s="5">
+      <c r="C108" s="4">
         <v>0.3</v>
       </c>
     </row>
-    <row r="109" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A109" s="15">
+    <row r="109" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A109" s="8">
         <v>44931.541666666664</v>
       </c>
-      <c r="B109" s="4">
+      <c r="B109" s="3">
         <v>2.1161480247286501E-4</v>
       </c>
-      <c r="C109" s="5">
+      <c r="C109" s="4">
         <v>0.2</v>
       </c>
     </row>
-    <row r="110" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A110" s="15">
+    <row r="110" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A110" s="8">
         <v>44931.583333333336</v>
       </c>
-      <c r="B110" s="4">
+      <c r="B110" s="3">
         <v>2.111316636544338E-4</v>
       </c>
-      <c r="C110" s="5">
+      <c r="C110" s="4">
         <v>0.1</v>
       </c>
     </row>
-    <row r="111" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A111" s="15">
+    <row r="111" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A111" s="8">
         <v>44931.625</v>
       </c>
-      <c r="B111" s="4">
+      <c r="B111" s="3">
         <v>2.154799130203146E-4</v>
       </c>
-      <c r="C111" s="5">
+      <c r="C111" s="4">
         <v>0.2</v>
       </c>
     </row>
-    <row r="112" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A112" s="15">
+    <row r="112" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A112" s="8">
         <v>44931.666666666664</v>
       </c>
-      <c r="B112" s="4">
+      <c r="B112" s="3">
         <v>2.2127757884148901E-4</v>
       </c>
-      <c r="C112" s="5">
+      <c r="C112" s="4">
         <v>0.3</v>
       </c>
     </row>
-    <row r="113" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A113" s="15">
+    <row r="113" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A113" s="8">
         <v>44931.708333333336</v>
       </c>
-      <c r="B113" s="4">
+      <c r="B113" s="3">
         <v>2.32389771665406E-4</v>
       </c>
-      <c r="C113" s="5">
+      <c r="C113" s="4">
         <v>0.4</v>
       </c>
     </row>
-    <row r="114" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A114" s="15">
+    <row r="114" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A114" s="8">
         <v>44931.75</v>
       </c>
-      <c r="B114" s="4">
+      <c r="B114" s="3">
         <v>2.4205254803403E-4</v>
       </c>
-      <c r="C114" s="5">
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="115" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A115" s="15">
+      <c r="C114" s="4">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="115" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A115" s="8">
         <v>44931.791666666664</v>
       </c>
-      <c r="B115" s="4">
+      <c r="B115" s="3">
         <v>2.4446824212618598E-4</v>
       </c>
-      <c r="C115" s="5">
+      <c r="C115" s="4">
         <v>0.6</v>
       </c>
     </row>
-    <row r="116" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A116" s="15">
+    <row r="116" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A116" s="8">
         <v>44931.833333333336</v>
       </c>
-      <c r="B116" s="4">
+      <c r="B116" s="3">
         <v>2.439851033077548E-4</v>
       </c>
-      <c r="C116" s="5">
+      <c r="C116" s="4">
         <v>0.7</v>
       </c>
     </row>
-    <row r="117" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A117" s="15">
+    <row r="117" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A117" s="8">
         <v>44931.875</v>
       </c>
-      <c r="B117" s="4">
+      <c r="B117" s="3">
         <v>2.3432232693913101E-4</v>
       </c>
-      <c r="C117" s="5">
+      <c r="C117" s="4">
         <v>0.6</v>
       </c>
     </row>
-    <row r="118" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A118" s="15">
+    <row r="118" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A118" s="8">
         <v>44931.916666666664</v>
       </c>
-      <c r="B118" s="4">
+      <c r="B118" s="3">
         <v>2.0774969192541539E-4</v>
       </c>
-      <c r="C118" s="5">
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="119" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A119" s="15">
+      <c r="C118" s="4">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="119" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A119" s="8">
         <v>44931.958333333336</v>
       </c>
-      <c r="B119" s="4">
+      <c r="B119" s="3">
         <v>1.492898948952402E-4</v>
       </c>
-      <c r="C119" s="5">
+      <c r="C119" s="4">
         <v>0.4</v>
       </c>
     </row>
-    <row r="120" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A120" s="15">
+    <row r="120" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A120" s="8">
         <v>44932</v>
       </c>
-      <c r="B120" s="4">
+      <c r="B120" s="3">
         <v>1.1885214933407501E-4</v>
       </c>
-      <c r="C120" s="5">
+      <c r="C120" s="4">
         <v>0.3</v>
       </c>
     </row>
-    <row r="121" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A121" s="15">
+    <row r="121" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A121" s="8">
         <v>44932.041666666664</v>
       </c>
-      <c r="B121" s="4">
+      <c r="B121" s="3">
         <v>1.17821643065071E-4</v>
       </c>
-      <c r="C121" s="5">
+      <c r="C121" s="4">
         <v>0.2</v>
       </c>
     </row>
-    <row r="122" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A122" s="15">
+    <row r="122" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A122" s="8">
         <v>44932.083333333336</v>
       </c>
-      <c r="B122" s="4">
+      <c r="B122" s="3">
         <v>1.21407519158355E-4</v>
       </c>
-      <c r="C122" s="5">
+      <c r="C122" s="4">
         <v>0.1</v>
       </c>
     </row>
-    <row r="123" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A123" s="15">
+    <row r="123" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A123" s="8">
         <v>44932.125</v>
       </c>
-      <c r="B123" s="4">
+      <c r="B123" s="3">
         <v>1.2448112723831341E-4</v>
       </c>
-      <c r="C123" s="5">
+      <c r="C123" s="4">
         <v>0.2</v>
       </c>
     </row>
-    <row r="124" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A124" s="15">
+    <row r="124" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A124" s="8">
         <v>44932.166666666664</v>
       </c>
-      <c r="B124" s="4">
+      <c r="B124" s="3">
         <v>1.342142194915152E-4</v>
       </c>
-      <c r="C124" s="5">
+      <c r="C124" s="4">
         <v>0.3</v>
       </c>
     </row>
-    <row r="125" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A125" s="15">
+    <row r="125" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A125" s="8">
         <v>44932.208333333336</v>
       </c>
-      <c r="B125" s="4">
+      <c r="B125" s="3">
         <v>1.598276201578344E-4</v>
       </c>
-      <c r="C125" s="5">
+      <c r="C125" s="4">
         <v>0.4</v>
       </c>
     </row>
-    <row r="126" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A126" s="15">
+    <row r="126" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A126" s="8">
         <v>44932.25</v>
       </c>
-      <c r="B126" s="4">
+      <c r="B126" s="3">
         <v>2.294960699702244E-4</v>
       </c>
-      <c r="C126" s="5">
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="127" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A127" s="15">
+      <c r="C126" s="4">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="127" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A127" s="8">
         <v>44932.291666666664</v>
       </c>
-      <c r="B127" s="4">
+      <c r="B127" s="3">
         <v>2.9557864368932879E-4</v>
       </c>
-      <c r="C127" s="5">
+      <c r="C127" s="4">
         <v>0.6</v>
       </c>
     </row>
-    <row r="128" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A128" s="15">
+    <row r="128" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A128" s="8">
         <v>44932.333333333336</v>
       </c>
-      <c r="B128" s="4">
+      <c r="B128" s="3">
         <v>2.7508792315627319E-4</v>
       </c>
-      <c r="C128" s="5">
+      <c r="C128" s="4">
         <v>0.7</v>
       </c>
     </row>
-    <row r="129" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A129" s="15">
+    <row r="129" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A129" s="8">
         <v>44932.375</v>
       </c>
-      <c r="B129" s="4">
+      <c r="B129" s="3">
         <v>2.6125668679646038E-4</v>
       </c>
-      <c r="C129" s="5">
+      <c r="C129" s="4">
         <v>0.6</v>
       </c>
     </row>
-    <row r="130" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A130" s="15">
+    <row r="130" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A130" s="8">
         <v>44932.416666666664</v>
       </c>
-      <c r="B130" s="4">
+      <c r="B130" s="3">
         <v>2.4998679050328002E-4</v>
       </c>
-      <c r="C130" s="5">
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="131" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A131" s="15">
+      <c r="C130" s="4">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="131" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A131" s="8">
         <v>44932.458333333336</v>
       </c>
-      <c r="B131" s="4">
+      <c r="B131" s="3">
         <v>2.3820462619677301E-4</v>
       </c>
-      <c r="C131" s="5">
+      <c r="C131" s="4">
         <v>0.4</v>
       </c>
     </row>
-    <row r="132" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A132" s="15">
+    <row r="132" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A132" s="8">
         <v>44932.5</v>
       </c>
-      <c r="B132" s="4">
+      <c r="B132" s="3">
         <v>2.294960699702244E-4</v>
       </c>
-      <c r="C132" s="5">
+      <c r="C132" s="4">
         <v>0.3</v>
       </c>
     </row>
-    <row r="133" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A133" s="15">
+    <row r="133" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A133" s="8">
         <v>44932.541666666664</v>
       </c>
-      <c r="B133" s="4">
+      <c r="B133" s="3">
         <v>2.243733898369602E-4</v>
       </c>
-      <c r="C133" s="5">
+      <c r="C133" s="4">
         <v>0.2</v>
       </c>
     </row>
-    <row r="134" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A134" s="15">
+    <row r="134" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A134" s="8">
         <v>44932.583333333336</v>
       </c>
-      <c r="B134" s="4">
+      <c r="B134" s="3">
         <v>2.23861121823634E-4</v>
       </c>
-      <c r="C134" s="5">
+      <c r="C134" s="4">
         <v>0.1</v>
       </c>
     </row>
-    <row r="135" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A135" s="15">
+    <row r="135" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A135" s="8">
         <v>44932.625</v>
       </c>
-      <c r="B135" s="4">
+      <c r="B135" s="3">
         <v>2.2847153394357119E-4</v>
       </c>
-      <c r="C135" s="5">
+      <c r="C135" s="4">
         <v>0.2</v>
       </c>
     </row>
-    <row r="136" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A136" s="15">
+    <row r="136" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A136" s="8">
         <v>44932.666666666664</v>
       </c>
-      <c r="B136" s="4">
+      <c r="B136" s="3">
         <v>2.34618750103488E-4</v>
       </c>
-      <c r="C136" s="5">
+      <c r="C136" s="4">
         <v>0.3</v>
       </c>
     </row>
-    <row r="137" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A137" s="15">
+    <row r="137" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A137" s="8">
         <v>44932.708333333336</v>
       </c>
-      <c r="B137" s="4">
+      <c r="B137" s="3">
         <v>2.4640091440999501E-4</v>
       </c>
-      <c r="C137" s="5">
+      <c r="C137" s="4">
         <v>0.4</v>
       </c>
     </row>
-    <row r="138" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A138" s="15">
+    <row r="138" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A138" s="8">
         <v>44932.75</v>
       </c>
-      <c r="B138" s="4">
+      <c r="B138" s="3">
         <v>2.5664627467652298E-4</v>
       </c>
-      <c r="C138" s="5">
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="139" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A139" s="15">
+      <c r="C138" s="4">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="139" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A139" s="8">
         <v>44932.791666666664</v>
       </c>
-      <c r="B139" s="4">
+      <c r="B139" s="3">
         <v>2.5920761474315499E-4</v>
       </c>
-      <c r="C139" s="5">
+      <c r="C139" s="4">
         <v>0.6</v>
       </c>
     </row>
-    <row r="140" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A140" s="15">
+    <row r="140" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A140" s="8">
         <v>44932.833333333336</v>
       </c>
-      <c r="B140" s="4">
+      <c r="B140" s="3">
         <v>2.5869534672982858E-4</v>
       </c>
-      <c r="C140" s="5">
+      <c r="C140" s="4">
         <v>0.7</v>
       </c>
     </row>
-    <row r="141" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A141" s="15">
+    <row r="141" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A141" s="8">
         <v>44932.875</v>
       </c>
-      <c r="B141" s="4">
+      <c r="B141" s="3">
         <v>2.4844998646330078E-4</v>
       </c>
-      <c r="C141" s="5">
+      <c r="C141" s="4">
         <v>0.6</v>
       </c>
     </row>
-    <row r="142" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A142" s="15">
+    <row r="142" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A142" s="8">
         <v>44932.916666666664</v>
       </c>
-      <c r="B142" s="4">
+      <c r="B142" s="3">
         <v>2.2027524573034921E-4</v>
       </c>
-      <c r="C142" s="5">
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="143" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A143" s="15">
+      <c r="C142" s="4">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="143" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A143" s="8">
         <v>44932.958333333336</v>
       </c>
-      <c r="B143" s="4">
+      <c r="B143" s="3">
         <v>1.5829081611785521E-4</v>
       </c>
-      <c r="C143" s="5">
+      <c r="C143" s="4">
         <v>0.4</v>
       </c>
     </row>
-    <row r="144" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A144" s="15">
+    <row r="144" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A144" s="8">
         <v>44933</v>
       </c>
-      <c r="B144" s="4">
+      <c r="B144" s="3">
         <v>1.260179312782926E-4</v>
       </c>
-      <c r="C144" s="5">
+      <c r="C144" s="4">
         <v>0.3</v>
       </c>
     </row>
-    <row r="145" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A145" s="15">
+    <row r="145" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A145" s="8">
         <v>44933.041666666664</v>
       </c>
-      <c r="B145" s="4">
+      <c r="B145" s="3">
         <v>1.265761578251604E-4</v>
       </c>
-      <c r="C145" s="5">
+      <c r="C145" s="4">
         <v>0.2</v>
       </c>
     </row>
-    <row r="146" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A146" s="15">
+    <row r="146" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A146" s="8">
         <v>44933.083333333336</v>
       </c>
-      <c r="B146" s="4">
+      <c r="B146" s="3">
         <v>1.304284756720128E-4</v>
       </c>
-      <c r="C146" s="5">
+      <c r="C146" s="4">
         <v>0.1</v>
       </c>
     </row>
-    <row r="147" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A147" s="15">
+    <row r="147" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A147" s="8">
         <v>44933.125</v>
       </c>
-      <c r="B147" s="4">
+      <c r="B147" s="3">
         <v>1.3373046239788678E-3</v>
       </c>
-      <c r="C147" s="5">
+      <c r="C147" s="4">
         <v>0.2</v>
       </c>
     </row>
-    <row r="148" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A148" s="15">
+    <row r="148" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A148" s="8">
         <v>44933.166666666664</v>
       </c>
-      <c r="B148" s="4">
+      <c r="B148" s="3">
         <v>1.441867536964872E-4</v>
       </c>
-      <c r="C148" s="5">
+      <c r="C148" s="4">
         <v>0.3</v>
       </c>
     </row>
-    <row r="149" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A149" s="15">
+    <row r="149" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A149" s="8">
         <v>44933.208333333336</v>
       </c>
-      <c r="B149" s="4">
+      <c r="B149" s="3">
         <v>1.7170330974543481E-4</v>
       </c>
-      <c r="C149" s="5">
+      <c r="C149" s="4">
         <v>0.4</v>
       </c>
     </row>
-    <row r="150" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A150" s="15">
+    <row r="150" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A150" s="8">
         <v>44933.25</v>
       </c>
-      <c r="B150" s="4">
+      <c r="B150" s="3">
         <v>2.46548342198573E-4</v>
       </c>
-      <c r="C150" s="5">
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="151" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A151" s="15">
+      <c r="C150" s="4">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="151" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A151" s="8">
         <v>44933.291666666664</v>
       </c>
-      <c r="B151" s="4">
+      <c r="B151" s="3">
         <v>3.1754105680485798E-4</v>
       </c>
-      <c r="C151" s="5">
+      <c r="C151" s="4">
         <v>0.6</v>
       </c>
     </row>
-    <row r="152" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A152" s="15">
+    <row r="152" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A152" s="8">
         <v>44933.333333333336</v>
       </c>
-      <c r="B152" s="4">
+      <c r="B152" s="3">
         <v>2.9552781196570021E-4</v>
       </c>
-      <c r="C152" s="5">
+      <c r="C152" s="4">
         <v>0.7</v>
       </c>
     </row>
-    <row r="153" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A153" s="15">
+    <row r="153" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A153" s="8">
         <v>44933.375</v>
       </c>
-      <c r="B153" s="4">
+      <c r="B153" s="3">
         <v>2.8066887169926841E-4</v>
       </c>
-      <c r="C153" s="5">
+      <c r="C153" s="4">
         <v>0.6</v>
       </c>
     </row>
-    <row r="154" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A154" s="15">
+    <row r="154" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A154" s="8">
         <v>44933.416666666664</v>
       </c>
-      <c r="B154" s="4">
+      <c r="B154" s="3">
         <v>2.6856158703773202E-4</v>
       </c>
-      <c r="C154" s="5">
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="155" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A155" s="15">
+      <c r="C154" s="4">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="155" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A155" s="8">
         <v>44933.458333333336</v>
       </c>
-      <c r="B155" s="4">
+      <c r="B155" s="3">
         <v>2.5590397125521518E-4</v>
       </c>
-      <c r="C155" s="5">
+      <c r="C155" s="4">
         <v>0.4</v>
       </c>
     </row>
-    <row r="156" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A156" s="15">
+    <row r="156" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A156" s="8">
         <v>44933.5</v>
       </c>
-      <c r="B156" s="4">
+      <c r="B156" s="3">
         <v>2.46548342198573E-4</v>
       </c>
-      <c r="C156" s="5">
+      <c r="C156" s="4">
         <v>0.3</v>
       </c>
     </row>
-    <row r="157" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A157" s="15">
+    <row r="157" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A157" s="8">
         <v>44933.541666666664</v>
       </c>
-      <c r="B157" s="4">
+      <c r="B157" s="3">
         <v>2.4104503098878341E-4</v>
       </c>
-      <c r="C157" s="5">
+      <c r="C157" s="4">
         <v>0.2</v>
       </c>
     </row>
-    <row r="158" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A158" s="15">
+    <row r="158" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A158" s="8">
         <v>44933.583333333336</v>
       </c>
-      <c r="B158" s="4">
+      <c r="B158" s="3">
         <v>2.4049469986780439E-4</v>
       </c>
-      <c r="C158" s="5">
+      <c r="C158" s="4">
         <v>0.1</v>
       </c>
     </row>
-    <row r="159" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A159" s="15">
+    <row r="159" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A159" s="8">
         <v>44933.625</v>
       </c>
-      <c r="B159" s="4">
+      <c r="B159" s="3">
         <v>2.4544767995661498E-4</v>
       </c>
-      <c r="C159" s="5">
+      <c r="C159" s="4">
         <v>0.2</v>
       </c>
     </row>
-    <row r="160" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A160" s="15">
+    <row r="160" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A160" s="8">
         <v>44933.666666666664</v>
       </c>
-      <c r="B160" s="4">
+      <c r="B160" s="3">
         <v>2.52051653408363E-4</v>
       </c>
-      <c r="C160" s="5">
+      <c r="C160" s="4">
         <v>0.3</v>
       </c>
     </row>
-    <row r="161" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A161" s="15">
+    <row r="161" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A161" s="8">
         <v>44933.708333333336</v>
       </c>
-      <c r="B161" s="4">
+      <c r="B161" s="3">
         <v>2.6470926919087859E-4</v>
       </c>
-      <c r="C161" s="5">
+      <c r="C161" s="4">
         <v>0.4</v>
       </c>
     </row>
-    <row r="162" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A162" s="15">
+    <row r="162" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A162" s="8">
         <v>44933.75</v>
       </c>
-      <c r="B162" s="4">
+      <c r="B162" s="3">
         <v>2.7571589161045799E-4</v>
       </c>
-      <c r="C162" s="5">
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="163" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A163" s="15">
+      <c r="C162" s="4">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="163" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A163" s="8">
         <v>44933.791666666664</v>
       </c>
-      <c r="B163" s="4">
+      <c r="B163" s="3">
         <v>2.7846754721535199E-4</v>
       </c>
-      <c r="C163" s="5">
+      <c r="C163" s="4">
         <v>0.6</v>
       </c>
     </row>
-    <row r="164" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A164" s="15">
+    <row r="164" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A164" s="8">
         <v>44933.833333333336</v>
       </c>
-      <c r="B164" s="4">
+      <c r="B164" s="3">
         <v>2.77917216094373E-4</v>
       </c>
-      <c r="C164" s="5">
+      <c r="C164" s="4">
         <v>0.7</v>
       </c>
     </row>
-    <row r="165" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A165" s="15">
+    <row r="165" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A165" s="8">
         <v>44933.875</v>
       </c>
-      <c r="B165" s="4">
+      <c r="B165" s="3">
         <v>2.6691059367479458E-4</v>
       </c>
-      <c r="C165" s="5">
+      <c r="C165" s="4">
         <v>0.6</v>
       </c>
     </row>
-    <row r="166" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A166" s="15">
+    <row r="166" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A166" s="8">
         <v>44933.916666666664</v>
       </c>
-      <c r="B166" s="4">
+      <c r="B166" s="3">
         <v>2.36642382020952E-4</v>
       </c>
-      <c r="C166" s="5">
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="167" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A167" s="15">
+      <c r="C166" s="4">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="167" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A167" s="8">
         <v>44933.958333333336</v>
       </c>
-      <c r="B167" s="4">
+      <c r="B167" s="3">
         <v>1.700523163824978E-4</v>
       </c>
-      <c r="C167" s="5">
+      <c r="C167" s="4">
         <v>0.4</v>
       </c>
     </row>
-    <row r="168" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A168" s="16">
+    <row r="168" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A168" s="9">
         <v>44934</v>
       </c>
-      <c r="B168" s="4">
+      <c r="B168" s="3">
         <v>1.5513902023694899E-4</v>
       </c>
-      <c r="C168" s="5">
+      <c r="C168" s="4">
         <v>0.3</v>
       </c>
     </row>
-    <row r="169" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A169" s="15">
+    <row r="169" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A169" s="8">
         <v>44934.041666666664</v>
       </c>
-      <c r="B169" s="4">
+      <c r="B169" s="3">
         <v>1.7170330974543481E-4</v>
       </c>
-      <c r="C169" s="5">
+      <c r="C169" s="4">
         <v>0.2</v>
       </c>
     </row>
-    <row r="170" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A170" s="16">
+    <row r="170" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A170" s="9">
         <v>44934.083333333336</v>
       </c>
-      <c r="B170" s="4">
+      <c r="B170" s="3">
         <v>2.46548342198573E-4</v>
       </c>
-      <c r="C170" s="5">
+      <c r="C170" s="4">
         <v>0.1</v>
       </c>
     </row>
-    <row r="171" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A171" s="15">
+    <row r="171" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A171" s="8">
         <v>44934.125</v>
       </c>
-      <c r="B171" s="4">
+      <c r="B171" s="3">
         <v>3.1754105680485798E-4</v>
       </c>
-      <c r="C171" s="5">
+      <c r="C171" s="4">
         <v>0.2</v>
       </c>
     </row>
-    <row r="172" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A172" s="16">
+    <row r="172" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A172" s="9">
         <v>44934.166666666664</v>
       </c>
-      <c r="B172" s="4">
+      <c r="B172" s="3">
         <v>2.9552781196570021E-4</v>
       </c>
-      <c r="C172" s="5">
+      <c r="C172" s="4">
         <v>0.3</v>
       </c>
     </row>
-    <row r="173" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A173" s="15">
+    <row r="173" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A173" s="8">
         <v>44934.208333333336</v>
       </c>
-      <c r="B173" s="4">
+      <c r="B173" s="3">
         <v>2.8066887169926841E-4</v>
       </c>
-      <c r="C173" s="5">
+      <c r="C173" s="4">
         <v>0.4</v>
       </c>
     </row>
-    <row r="174" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A174" s="16">
+    <row r="174" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A174" s="9">
         <v>44934.25</v>
       </c>
-      <c r="B174" s="4">
+      <c r="B174" s="3">
         <v>2.6856158703773202E-4</v>
       </c>
-      <c r="C174" s="5">
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="175" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A175" s="15">
+      <c r="C174" s="4">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="175" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A175" s="8">
         <v>44934.291666666664</v>
       </c>
-      <c r="B175" s="4">
+      <c r="B175" s="3">
         <v>2.5590397125521518E-4</v>
       </c>
-      <c r="C175" s="5">
+      <c r="C175" s="4">
         <v>0.6</v>
       </c>
     </row>
-    <row r="176" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A176" s="16">
+    <row r="176" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A176" s="9">
         <v>44934.333333333336</v>
       </c>
-      <c r="B176" s="4">
+      <c r="B176" s="3">
         <v>2.46548342198573E-4</v>
       </c>
-      <c r="C176" s="5">
+      <c r="C176" s="4">
         <v>0.7</v>
       </c>
     </row>
-    <row r="177" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A177" s="15">
+    <row r="177" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A177" s="8">
         <v>44934.375</v>
       </c>
-      <c r="B177" s="4">
+      <c r="B177" s="3">
         <v>2.4104503098878341E-4</v>
       </c>
-      <c r="C177" s="5">
+      <c r="C177" s="4">
         <v>0.6</v>
       </c>
     </row>
-    <row r="178" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A178" s="15">
+    <row r="178" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A178" s="8">
         <v>44933.958333333336</v>
       </c>
-      <c r="B178" s="4">
+      <c r="B178" s="3">
         <v>2.4049469986780439E-4</v>
       </c>
-      <c r="C178" s="5">
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="179" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A179" s="16">
+      <c r="C178" s="4">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="179" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A179" s="9">
         <v>44934</v>
       </c>
-      <c r="B179" s="4">
+      <c r="B179" s="3">
         <v>2.4544767995661498E-4</v>
       </c>
-      <c r="C179" s="5">
+      <c r="C179" s="4">
         <v>0.4</v>
       </c>
     </row>
-    <row r="180" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A180" s="15">
+    <row r="180" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A180" s="8">
         <v>44934.041666666664</v>
       </c>
-      <c r="B180" s="4">
+      <c r="B180" s="3">
         <v>2.52051653408363E-4</v>
       </c>
-      <c r="C180" s="5">
+      <c r="C180" s="4">
         <v>0.3</v>
       </c>
     </row>
-    <row r="181" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A181" s="16">
+    <row r="181" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A181" s="9">
         <v>44934.083333333336</v>
       </c>
-      <c r="B181" s="4">
+      <c r="B181" s="3">
         <v>2.6470926919087859E-4</v>
       </c>
-      <c r="C181" s="5">
+      <c r="C181" s="4">
         <v>0.2</v>
       </c>
     </row>
-    <row r="182" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A182" s="15">
+    <row r="182" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A182" s="8">
         <v>44934.125</v>
       </c>
-      <c r="B182" s="4">
+      <c r="B182" s="3">
         <v>2.7571589161045799E-4</v>
       </c>
-      <c r="C182" s="5">
+      <c r="C182" s="4">
         <v>0.1</v>
       </c>
     </row>
-    <row r="183" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A183" s="16">
+    <row r="183" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A183" s="9">
         <v>44934.166666666664</v>
       </c>
-      <c r="B183" s="4">
+      <c r="B183" s="3">
         <v>2.7846754721535199E-4</v>
       </c>
-      <c r="C183" s="5">
+      <c r="C183" s="4">
         <v>0.2</v>
       </c>
     </row>
-    <row r="184" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A184" s="15">
+    <row r="184" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A184" s="8">
         <v>44934.208333333336</v>
       </c>
-      <c r="B184" s="4">
+      <c r="B184" s="3">
         <v>2.77917216094373E-4</v>
       </c>
-      <c r="C184" s="5">
+      <c r="C184" s="4">
         <v>0.3</v>
       </c>
     </row>
-    <row r="185" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A185" s="16">
+    <row r="185" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A185" s="9">
         <v>44934.25</v>
       </c>
-      <c r="B185" s="4">
+      <c r="B185" s="3">
         <v>2.6691059367479458E-4</v>
       </c>
-      <c r="C185" s="5">
+      <c r="C185" s="4">
         <v>0.4</v>
       </c>
     </row>
-    <row r="186" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A186" s="15">
+    <row r="186" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A186" s="8">
         <v>44934.291666666664</v>
       </c>
-      <c r="B186" s="4">
+      <c r="B186" s="3">
         <v>2.36642382020952E-4</v>
       </c>
-      <c r="C186" s="5">
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="187" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A187" s="16">
+      <c r="C186" s="4">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="187" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A187" s="9">
         <v>44934.333333333336</v>
       </c>
-      <c r="B187" s="4">
+      <c r="B187" s="3">
         <v>1.700523163824978E-4</v>
       </c>
-      <c r="C187" s="5">
+      <c r="C187" s="4">
         <v>0.6</v>
       </c>
     </row>
-    <row r="188" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A188" s="15">
+    <row r="188" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A188" s="8">
         <v>44934.375</v>
       </c>
-      <c r="B188" s="4">
+      <c r="B188" s="3">
         <v>1.5513902023694899E-4</v>
       </c>
-      <c r="C188" s="5">
+      <c r="C188" s="4">
         <v>0.7</v>
       </c>
     </row>
-    <row r="189" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A189" s="15">
+    <row r="189" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A189" s="8">
         <v>44933.958333333336</v>
       </c>
-      <c r="B189" s="4">
+      <c r="B189" s="3">
         <v>1.7170330974543481E-4</v>
       </c>
-      <c r="C189" s="5">
+      <c r="C189" s="4">
         <v>0.6</v>
       </c>
     </row>
-    <row r="190" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A190" s="16">
+    <row r="190" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A190" s="9">
         <v>44934</v>
       </c>
-      <c r="B190" s="4">
+      <c r="B190" s="3">
         <v>2.46548342198573E-4</v>
       </c>
-      <c r="C190" s="5">
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="191" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A191" s="15">
+      <c r="C190" s="4">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="191" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A191" s="8">
         <v>44934.041666666664</v>
       </c>
-      <c r="B191" s="4">
+      <c r="B191" s="3">
         <v>3.1754105680485798E-4</v>
       </c>
-      <c r="C191" s="5">
+      <c r="C191" s="4">
         <v>0.4</v>
       </c>
     </row>
-    <row r="192" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A192" s="16">
+    <row r="192" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A192" s="9">
         <v>44934.083333333336</v>
       </c>
-      <c r="B192" s="4">
+      <c r="B192" s="3">
         <v>2.9552781196570021E-4</v>
       </c>
-      <c r="C192" s="5">
+      <c r="C192" s="4">
         <v>0.3</v>
       </c>
     </row>
-    <row r="193" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A193" s="16">
+    <row r="193" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A193" s="9">
         <v>44935.083333333336</v>
       </c>
-      <c r="B193" s="4">
+      <c r="B193" s="3">
         <v>2.8066887169926841E-4</v>
       </c>
-      <c r="C193" s="5">
+      <c r="C193" s="4">
         <v>0.2</v>
       </c>
     </row>
-    <row r="194" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A194" s="16">
+    <row r="194" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A194" s="9">
         <v>44936.083333333336</v>
       </c>
-      <c r="B194" s="4">
+      <c r="B194" s="3">
         <v>2.6856158703773202E-4</v>
       </c>
-      <c r="C194" s="5">
+      <c r="C194" s="4">
         <v>0.1</v>
       </c>
     </row>
-    <row r="195" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A195" s="16">
+    <row r="195" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A195" s="9">
         <v>44937.083333333336</v>
       </c>
-      <c r="B195" s="4">
+      <c r="B195" s="3">
         <v>2.5590397125521518E-4</v>
       </c>
-      <c r="C195" s="5">
+      <c r="C195" s="4">
         <v>0.2</v>
       </c>
     </row>
-    <row r="196" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A196" s="16">
+    <row r="196" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A196" s="9">
         <v>44938.083333333336</v>
       </c>
-      <c r="B196" s="4">
+      <c r="B196" s="3">
         <v>2.46548342198573E-4</v>
       </c>
-      <c r="C196" s="5">
+      <c r="C196" s="4">
         <v>0.3</v>
       </c>
     </row>
-    <row r="197" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A197" s="16">
+    <row r="197" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A197" s="9">
         <v>44939.083333333336</v>
       </c>
-      <c r="B197" s="4">
+      <c r="B197" s="3">
         <v>2.4104503098878341E-4</v>
       </c>
-      <c r="C197" s="5">
+      <c r="C197" s="4">
         <v>0.4</v>
       </c>
     </row>
-    <row r="198" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A198" s="16">
+    <row r="198" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A198" s="9">
         <v>44940.083333333336</v>
       </c>
-      <c r="B198" s="4">
+      <c r="B198" s="3">
         <v>2.4049469986780439E-4</v>
       </c>
-      <c r="C198" s="5">
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="199" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A199" s="16">
+      <c r="C198" s="4">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="199" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A199" s="9">
         <v>44941.083333333336</v>
       </c>
-      <c r="B199" s="4">
+      <c r="B199" s="3">
         <v>2.4544767995661498E-4</v>
       </c>
-      <c r="C199" s="5">
+      <c r="C199" s="4">
         <v>0.6</v>
       </c>
     </row>
-    <row r="200" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A200" s="16">
+    <row r="200" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A200" s="9">
         <v>44942.083333333336</v>
       </c>
-      <c r="B200" s="4">
+      <c r="B200" s="3">
         <v>2.52051653408363E-4</v>
       </c>
-      <c r="C200" s="5">
+      <c r="C200" s="4">
         <v>0.7</v>
       </c>
     </row>
-    <row r="201" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A201" s="16">
+    <row r="201" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A201" s="9">
         <v>44943.083333333336</v>
       </c>
-      <c r="B201" s="4">
+      <c r="B201" s="3">
         <v>2.6470926919087859E-4</v>
       </c>
-      <c r="C201" s="5">
+      <c r="C201" s="4">
         <v>0.6</v>
       </c>
     </row>
-    <row r="202" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A202" s="16">
+    <row r="202" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A202" s="9">
         <v>44944.083333333336</v>
       </c>
-      <c r="B202" s="4">
+      <c r="B202" s="3">
         <v>2.7571589161045799E-4</v>
       </c>
-      <c r="C202" s="5">
-        <v>0.5</v>
-      </c>
-    </row>
-    <row r="203" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A203" s="16">
+      <c r="C202" s="4">
+        <v>0.5</v>
+      </c>
+    </row>
+    <row r="203" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A203" s="9">
         <v>44945.083333333336</v>
       </c>
-      <c r="B203" s="4">
+      <c r="B203" s="3">
         <v>2.7846754721535199E-4</v>
       </c>
-      <c r="C203" s="5">
+      <c r="C203" s="4">
         <v>0.4</v>
       </c>
     </row>
-    <row r="204" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A204" s="16">
+    <row r="204" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A204" s="9">
         <v>44946.083333333336</v>
       </c>
-      <c r="B204" s="4">
+      <c r="B204" s="3">
         <v>2.77917216094373E-4</v>
       </c>
-      <c r="C204" s="5">
+      <c r="C204" s="4">
         <v>0.3</v>
       </c>
     </row>
-    <row r="205" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A205" s="16">
+    <row r="205" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A205" s="9">
         <v>44947.083333333336</v>
       </c>
-      <c r="B205" s="4">
+      <c r="B205" s="3">
         <v>2.6691059367479458E-4</v>
       </c>
-      <c r="C205" s="5">
+      <c r="C205" s="4">
         <v>0.2</v>
       </c>
     </row>
-    <row r="206" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A206" s="16">
+    <row r="206" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A206" s="9">
         <v>44948.083333333336</v>
       </c>
-      <c r="B206" s="4">
+      <c r="B206" s="3">
         <v>2.36642382020952E-4</v>
       </c>
-      <c r="C206" s="5">
+      <c r="C206" s="4">
         <v>0.1</v>
       </c>
     </row>
-    <row r="207" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A207" s="16">
+    <row r="207" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A207" s="9">
         <v>44949.083333333336</v>
       </c>
-      <c r="B207" s="4">
+      <c r="B207" s="3">
         <v>1.700523163824978E-4</v>
       </c>
-      <c r="C207" s="17">
+      <c r="C207" s="10">
         <v>0.2</v>
       </c>
     </row>
-    <row r="208" spans="1:3" x14ac:dyDescent="0.3">
-      <c r="A208" s="16">
+    <row r="208" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A208" s="9">
         <v>44950.083333333336</v>
       </c>
-      <c r="B208" s="4">
+      <c r="B208" s="3">
         <v>1.5513902023694899E-4</v>
       </c>
-      <c r="C208" s="17">
+      <c r="C208" s="10">
         <v>0.3</v>
       </c>
     </row>

</xml_diff>